<commit_message>
Rework spreadsheet keyed on workgroup; language derived, not audited per-mockup
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014BTMoKe4qeivFFNX4KkDkH
</commit_message>
<xml_diff>
--- a/_audit/Системные_сообщения_таблица.xlsx
+++ b/_audit/Системные_сообщения_таблица.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сводка" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Сообщения'!$A$1:$I$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Сообщения'!$A$1:$J$39</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -48,7 +48,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -63,6 +63,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDEDED"/>
       </patternFill>
     </fill>
     <fill>
@@ -102,7 +107,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -119,11 +124,15 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -490,18 +499,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="44" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -532,20 +542,25 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Язык</t>
+          <t>Воркгруппа (страна/регион)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Ожидаемый язык (по воркгруппе)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Статус контента</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Статус (что делать)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Комментарий</t>
         </is>
@@ -574,27 +589,32 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Первый вход (Бразилия), возраст не подтверждён</t>
+          <t>Первый вход, возраст не подтверждён</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Заглушка-ключ</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>Нет текста (заглушка)</t>
-        </is>
-      </c>
-      <c r="H2" s="4" t="inlineStr">
+          <t>SIGAP_BRAZIL</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Português (pt-BR)</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>i18n-ключ</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>Уточнить у разработки</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Нужен реальный текст на всех языках</t>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Текст локализуется по воркгруппе; запросить реальную формулировку</t>
         </is>
       </c>
     </row>
@@ -626,22 +646,27 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Заглушка-ключ</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>Нет текста (заглушка)</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
+          <t>SIGAP_BRAZIL</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Português (pt-BR)</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>i18n-ключ</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>Уточнить у разработки</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Мягкое предупреждение перед жёсткой блокировкой</t>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Запросить реальную формулировку</t>
         </is>
       </c>
     </row>
@@ -673,22 +698,27 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Заглушка-ключ</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>Нет текста (заглушка)</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
+          <t>SIGAP_BRAZIL</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Português (pt-BR)</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>i18n-ключ</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>Уточнить у разработки</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>Критично: окно без выхода, нужен выверенный текст</t>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Критично (окно без выхода); запросить выверенный текст</t>
         </is>
       </c>
     </row>
@@ -720,22 +750,27 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Заглушка-ключ</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>Нет текста (заглушка)</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
+          <t>NONE_MEXICO</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Español (es-MX)</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>i18n-ключ</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>Уточнить у разработки</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>В документе мало деталей по поведению</t>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Мало деталей по поведению; запросить текст</t>
         </is>
       </c>
     </row>
@@ -767,22 +802,27 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Заглушка-ключ</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>Нет текста (заглушка)</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
+          <t>SIGAP_BRAZIL</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Português (pt-BR)</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>i18n-ключ</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>Уточнить у разработки</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>Нужен реальный текст</t>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Запросить реальную формулировку</t>
         </is>
       </c>
     </row>
@@ -814,22 +854,27 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Заглушка-ключ</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>Нет текста (заглушка)</t>
-        </is>
-      </c>
-      <c r="H7" s="4" t="inlineStr">
+          <t>SIGAP_BRAZIL</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Português (pt-BR)</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>i18n-ключ</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>Уточнить у разработки</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>Нужен реальный текст</t>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Запросить реальную формулировку</t>
         </is>
       </c>
     </row>
@@ -861,20 +906,25 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Заглушка-ключ</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>Нет текста (заглушка)</t>
-        </is>
-      </c>
-      <c r="H8" s="4" t="inlineStr">
+          <t>SIGAP_BRAZIL</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Português (pt-BR)</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>i18n-ключ</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
         <is>
           <t>Уточнить у разработки</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>Многошаговый флоу — шаги и кнопки не ясны</t>
         </is>
@@ -908,22 +958,27 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>EN</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
+          <t>BCE</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>❓ уточнить (BCE)</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>Вшит в код</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="I9" s="5" t="inlineStr">
         <is>
           <t>Требует правок</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>Только EN и вшит в код — без разработки не перевести</t>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Текст вшит в код → НЕ переключает язык по воркгруппе. Вынести в локализацию (задача разработки)</t>
         </is>
       </c>
     </row>
@@ -950,27 +1005,32 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Сразу после регистрации (не Бразилия)</t>
+          <t>Сразу после регистрации</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
+          <t>Все, кроме Бразилии</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Все локали, кроме PT</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
         <is>
           <t>Вшит в код</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
+      <c r="I10" s="5" t="inlineStr">
         <is>
           <t>Требует правок</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>Только ES, вшит в код, конкурирует с другими окнами</t>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Вшит в код → один язык на все страны. Вынести в локализацию. Плюс конкуренция окон после рег</t>
         </is>
       </c>
     </row>
@@ -1002,22 +1062,27 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Заглушка-ключ</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>Нет текста (заглушка)</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
+          <t>Все</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Все активные локали</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>i18n-ключ</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
         <is>
           <t>Уточнить у разработки</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>Нужен реальный текст</t>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Запросить реальную формулировку</t>
         </is>
       </c>
     </row>
@@ -1049,22 +1114,27 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>EN</t>
-        </is>
-      </c>
-      <c r="G12" s="4" t="inlineStr">
+          <t>SIGAP_BRAZIL</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Português (pt-BR)</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
         <is>
           <t>Вшит в код</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr">
+      <c r="I12" s="5" t="inlineStr">
         <is>
           <t>Требует правок</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>Только EN для бразильской аудитории — нужен перевод</t>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Вшит в код → не подхватит PT по воркгруппе. Вынести в локализацию</t>
         </is>
       </c>
     </row>
@@ -1096,22 +1166,27 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Заглушка-ключ</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>Нет текста (заглушка)</t>
-        </is>
-      </c>
-      <c r="H13" s="4" t="inlineStr">
+          <t>SIGAP_BRAZIL</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Português (pt-BR)</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>i18n-ключ</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
         <is>
           <t>Уточнить у разработки</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>Обязательное окно, нужен реальный текст</t>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Обязательное окно; запросить реальную формулировку</t>
         </is>
       </c>
     </row>
@@ -1143,22 +1218,27 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>EN</t>
-        </is>
-      </c>
-      <c r="G14" s="4" t="inlineStr">
+          <t>Все</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Все активные локали</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
         <is>
           <t>Вшит в код</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr">
+      <c r="I14" s="5" t="inlineStr">
         <is>
           <t>Требует правок</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>EN; дублирует «уровень» из первого бонуса на другом языке</t>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Вшит в код → один язык на все страны. Дублирует «уровень» из M-09</t>
         </is>
       </c>
     </row>
@@ -1190,22 +1270,27 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>EN</t>
-        </is>
-      </c>
-      <c r="G15" s="4" t="inlineStr">
+          <t>Все</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Все активные локали</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
         <is>
           <t>Вшит в код</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr">
+      <c r="I15" s="5" t="inlineStr">
         <is>
           <t>Требует правок</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>Только EN</t>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Вшит в код → вынести в локализацию</t>
         </is>
       </c>
     </row>
@@ -1237,22 +1322,27 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>EN</t>
-        </is>
-      </c>
-      <c r="G16" s="4" t="inlineStr">
+          <t>Все</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Все активные локали</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
         <is>
           <t>Вшит в код</t>
         </is>
       </c>
-      <c r="H16" s="3" t="inlineStr">
+      <c r="I16" s="5" t="inlineStr">
         <is>
           <t>Требует правок</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>Только EN</t>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Вшит в код → вынести в локализацию</t>
         </is>
       </c>
     </row>
@@ -1284,22 +1374,27 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>EN</t>
-        </is>
-      </c>
-      <c r="G17" s="4" t="inlineStr">
+          <t>Все</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Все активные локали</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
         <is>
           <t>Вшит в код</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr">
+      <c r="I17" s="5" t="inlineStr">
         <is>
           <t>Требует правок</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
-        <is>
-          <t>Только EN</t>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Вшит в код → вынести в локализацию</t>
         </is>
       </c>
     </row>
@@ -1331,22 +1426,27 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>EN</t>
-        </is>
-      </c>
-      <c r="G18" s="4" t="inlineStr">
+          <t>Все</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Все активные локали</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
         <is>
           <t>Вшит в код</t>
         </is>
       </c>
-      <c r="H18" s="3" t="inlineStr">
+      <c r="I18" s="5" t="inlineStr">
         <is>
           <t>Требует правок</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>Только EN</t>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Вшит в код → вынести в локализацию</t>
         </is>
       </c>
     </row>
@@ -1378,22 +1478,27 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="inlineStr">
+          <t>Все</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Все активные локали</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
         <is>
           <t>Нет данных</t>
         </is>
       </c>
-      <c r="H19" s="4" t="inlineStr">
+      <c r="I19" s="4" t="inlineStr">
         <is>
           <t>Уточнить у разработки</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>Текст и кнопки в документе не описаны</t>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Текст и кнопки в источниках не описаны</t>
         </is>
       </c>
     </row>
@@ -1425,22 +1530,27 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>EN</t>
-        </is>
-      </c>
-      <c r="G20" s="4" t="inlineStr">
+          <t>Все</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Все активные локали</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
         <is>
           <t>Вшит в код</t>
         </is>
       </c>
-      <c r="H20" s="3" t="inlineStr">
+      <c r="I20" s="5" t="inlineStr">
         <is>
           <t>Требует правок</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>Только EN</t>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Вшит в код → вынести в локализацию</t>
         </is>
       </c>
     </row>
@@ -1472,22 +1582,27 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>EN</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
+          <t>Все</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Все активные локали</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
         <is>
           <t>Вшит в код</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr">
+      <c r="I21" s="5" t="inlineStr">
         <is>
           <t>Требует правок</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
-        <is>
-          <t>EN; встречается под двумя именами — возможно дубль</t>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Вшит в код → вынести в локализацию. Встречается под двумя именами — возможно дубль</t>
         </is>
       </c>
     </row>
@@ -1519,22 +1634,27 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>PT</t>
-        </is>
-      </c>
-      <c r="G22" s="5" t="inlineStr">
+          <t>❓ уточнить</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>зависит от воркгруппы</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
         <is>
           <t>Текст есть</t>
         </is>
       </c>
-      <c r="H22" s="3" t="inlineStr">
-        <is>
-          <t>Требует правок</t>
-        </is>
-      </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>Только PT</t>
+      <c r="I22" s="4" t="inlineStr">
+        <is>
+          <t>Уточнить у разработки</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Плашки нет в дев-документации — подтвердить воркгруппу</t>
         </is>
       </c>
     </row>
@@ -1566,22 +1686,27 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>PT</t>
-        </is>
-      </c>
-      <c r="G23" s="5" t="inlineStr">
+          <t>❓ уточнить</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>зависит от воркгруппы</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="inlineStr">
         <is>
           <t>Текст есть</t>
         </is>
       </c>
-      <c r="H23" s="3" t="inlineStr">
-        <is>
-          <t>Требует правок</t>
-        </is>
-      </c>
-      <c r="I23" s="2" t="inlineStr">
-        <is>
-          <t>Только PT</t>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>Уточнить у разработки</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Плашки нет в дев-документации — подтвердить воркгруппу</t>
         </is>
       </c>
     </row>
@@ -1613,22 +1738,27 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>PT</t>
-        </is>
-      </c>
-      <c r="G24" s="5" t="inlineStr">
+          <t>❓ уточнить</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>зависит от воркгруппы</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
         <is>
           <t>Текст есть</t>
         </is>
       </c>
-      <c r="H24" s="3" t="inlineStr">
-        <is>
-          <t>Требует правок</t>
-        </is>
-      </c>
-      <c r="I24" s="2" t="inlineStr">
-        <is>
-          <t>Только PT</t>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t>Уточнить у разработки</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Плашки нет в дев-документации — подтвердить воркгруппу</t>
         </is>
       </c>
     </row>
@@ -1660,22 +1790,27 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>EN</t>
-        </is>
-      </c>
-      <c r="G25" s="5" t="inlineStr">
+          <t>❓ уточнить</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>зависит от воркгруппы</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr">
         <is>
           <t>Текст есть</t>
         </is>
       </c>
-      <c r="H25" s="3" t="inlineStr">
+      <c r="I25" s="5" t="inlineStr">
         <is>
           <t>Требует правок</t>
         </is>
       </c>
-      <c r="I25" s="2" t="inlineStr">
-        <is>
-          <t>Успех помечен оранжевой иконкой предупреждения</t>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>Успех помечен оранжевой иконкой предупреждения (цвет/иконка)</t>
         </is>
       </c>
     </row>
@@ -1707,20 +1842,25 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>EN</t>
-        </is>
-      </c>
-      <c r="G26" s="5" t="inlineStr">
+          <t>❓ уточнить</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>зависит от воркгруппы</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr">
         <is>
           <t>Текст есть</t>
         </is>
       </c>
-      <c r="H26" s="5" t="inlineStr">
+      <c r="I26" s="6" t="inlineStr">
         <is>
           <t>ОК</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr">
+      <c r="J26" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1754,22 +1894,27 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>EN</t>
-        </is>
-      </c>
-      <c r="G27" s="5" t="inlineStr">
+          <t>❓ уточнить</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>зависит от воркгруппы</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="inlineStr">
         <is>
           <t>Текст есть</t>
         </is>
       </c>
-      <c r="H27" s="3" t="inlineStr">
+      <c r="I27" s="5" t="inlineStr">
         <is>
           <t>Требует правок</t>
         </is>
       </c>
-      <c r="I27" s="2" t="inlineStr">
-        <is>
-          <t>Формулировка-команда вместо факта («Удалено»)</t>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>Формулировка-команда вместо факта («Удалено из избранного»)</t>
         </is>
       </c>
     </row>
@@ -1801,22 +1946,27 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>PT</t>
-        </is>
-      </c>
-      <c r="G28" s="5" t="inlineStr">
+          <t>❓ уточнить</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>зависит от воркгруппы</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr">
         <is>
           <t>Текст есть</t>
         </is>
       </c>
-      <c r="H28" s="3" t="inlineStr">
-        <is>
-          <t>Требует правок</t>
-        </is>
-      </c>
-      <c r="I28" s="2" t="inlineStr">
-        <is>
-          <t>Только PT</t>
+      <c r="I28" s="6" t="inlineStr">
+        <is>
+          <t>ОК</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1848,22 +1998,27 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>PT</t>
-        </is>
-      </c>
-      <c r="G29" s="5" t="inlineStr">
+          <t>❓ уточнить</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>зависит от воркгруппы</t>
+        </is>
+      </c>
+      <c r="H29" s="6" t="inlineStr">
         <is>
           <t>Текст есть</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr">
+      <c r="I29" s="5" t="inlineStr">
         <is>
           <t>Требует правок</t>
         </is>
       </c>
-      <c r="I29" s="2" t="inlineStr">
-        <is>
-          <t>Помечено warning, хотя это error; только PT</t>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>Помечено как предупреждение, хотя это ошибка (цвет/иконка)</t>
         </is>
       </c>
     </row>
@@ -1895,22 +2050,27 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>EN</t>
-        </is>
-      </c>
-      <c r="G30" s="5" t="inlineStr">
+          <t>❓ уточнить</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>зависит от воркгруппы</t>
+        </is>
+      </c>
+      <c r="H30" s="6" t="inlineStr">
         <is>
           <t>Текст есть</t>
         </is>
       </c>
-      <c r="H30" s="3" t="inlineStr">
-        <is>
-          <t>Требует правок</t>
-        </is>
-      </c>
-      <c r="I30" s="2" t="inlineStr">
-        <is>
-          <t>Консистентность языка с PT-сообщениями</t>
+      <c r="I30" s="6" t="inlineStr">
+        <is>
+          <t>ОК</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1942,22 +2102,27 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="G31" s="5" t="inlineStr">
+          <t>❓ уточнить</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>зависит от воркгруппы</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr">
         <is>
           <t>Текст есть</t>
         </is>
       </c>
-      <c r="H31" s="3" t="inlineStr">
-        <is>
-          <t>Требует правок</t>
-        </is>
-      </c>
-      <c r="I31" s="2" t="inlineStr">
-        <is>
-          <t>Только ES</t>
+      <c r="I31" s="6" t="inlineStr">
+        <is>
+          <t>ОК</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1989,22 +2154,27 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>PT</t>
-        </is>
-      </c>
-      <c r="G32" s="5" t="inlineStr">
+          <t>❓ уточнить</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>зависит от воркгруппы</t>
+        </is>
+      </c>
+      <c r="H32" s="6" t="inlineStr">
         <is>
           <t>Текст есть</t>
         </is>
       </c>
-      <c r="H32" s="3" t="inlineStr">
+      <c r="I32" s="5" t="inlineStr">
         <is>
           <t>Требует правок</t>
         </is>
       </c>
-      <c r="I32" s="2" t="inlineStr">
-        <is>
-          <t>Дублирует тему окна лимитов</t>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>Та же тема, что окно лимитов — дублирование канала, свести тон</t>
         </is>
       </c>
     </row>
@@ -2036,22 +2206,27 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>PT</t>
-        </is>
-      </c>
-      <c r="G33" s="5" t="inlineStr">
+          <t>❓ уточнить</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>зависит от воркгруппы</t>
+        </is>
+      </c>
+      <c r="H33" s="6" t="inlineStr">
         <is>
           <t>Текст есть</t>
         </is>
       </c>
-      <c r="H33" s="3" t="inlineStr">
+      <c r="I33" s="5" t="inlineStr">
         <is>
           <t>Требует правок</t>
         </is>
       </c>
-      <c r="I33" s="2" t="inlineStr">
-        <is>
-          <t>Дублирует тему окна лимитов</t>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>Та же тема, что окно лимитов — дублирование канала, свести тон</t>
         </is>
       </c>
     </row>
@@ -2083,20 +2258,25 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>EN</t>
-        </is>
-      </c>
-      <c r="G34" s="5" t="inlineStr">
+          <t>❓ уточнить</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>зависит от воркгруппы</t>
+        </is>
+      </c>
+      <c r="H34" s="6" t="inlineStr">
         <is>
           <t>Текст есть</t>
         </is>
       </c>
-      <c r="H34" s="5" t="inlineStr">
+      <c r="I34" s="6" t="inlineStr">
         <is>
           <t>ОК</t>
         </is>
       </c>
-      <c r="I34" s="2" t="inlineStr">
+      <c r="J34" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2130,22 +2310,27 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>EN</t>
-        </is>
-      </c>
-      <c r="G35" s="5" t="inlineStr">
+          <t>❓ уточнить</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>зависит от воркгруппы</t>
+        </is>
+      </c>
+      <c r="H35" s="6" t="inlineStr">
         <is>
           <t>Текст есть</t>
         </is>
       </c>
-      <c r="H35" s="3" t="inlineStr">
+      <c r="I35" s="5" t="inlineStr">
         <is>
           <t>Требует правок</t>
         </is>
       </c>
-      <c r="I35" s="2" t="inlineStr">
-        <is>
-          <t>Негатив с зелёной иконкой успеха</t>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>Негатив с зелёной иконкой успеха (цвет/иконка)</t>
         </is>
       </c>
     </row>
@@ -2177,20 +2362,25 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>EN</t>
-        </is>
-      </c>
-      <c r="G36" s="5" t="inlineStr">
+          <t>❓ уточнить</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>зависит от воркгруппы</t>
+        </is>
+      </c>
+      <c r="H36" s="6" t="inlineStr">
         <is>
           <t>Текст есть</t>
         </is>
       </c>
-      <c r="H36" s="5" t="inlineStr">
+      <c r="I36" s="6" t="inlineStr">
         <is>
           <t>ОК</t>
         </is>
       </c>
-      <c r="I36" s="2" t="inlineStr">
+      <c r="J36" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2224,22 +2414,27 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>PT</t>
-        </is>
-      </c>
-      <c r="G37" s="5" t="inlineStr">
+          <t>❓ уточнить</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>зависит от воркгруппы</t>
+        </is>
+      </c>
+      <c r="H37" s="6" t="inlineStr">
         <is>
           <t>Текст есть</t>
         </is>
       </c>
-      <c r="H37" s="3" t="inlineStr">
-        <is>
-          <t>Требует правок</t>
-        </is>
-      </c>
-      <c r="I37" s="2" t="inlineStr">
-        <is>
-          <t>Только PT</t>
+      <c r="I37" s="6" t="inlineStr">
+        <is>
+          <t>ОК</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -2271,20 +2466,25 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>EN</t>
-        </is>
-      </c>
-      <c r="G38" s="5" t="inlineStr">
+          <t>❓ уточнить</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>зависит от воркгруппы</t>
+        </is>
+      </c>
+      <c r="H38" s="6" t="inlineStr">
         <is>
           <t>Текст есть</t>
         </is>
       </c>
-      <c r="H38" s="5" t="inlineStr">
+      <c r="I38" s="6" t="inlineStr">
         <is>
           <t>ОК</t>
         </is>
       </c>
-      <c r="I38" s="2" t="inlineStr">
+      <c r="J38" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2318,27 +2518,32 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>EN</t>
-        </is>
-      </c>
-      <c r="G39" s="5" t="inlineStr">
+          <t>❓ уточнить</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>зависит от воркгруппы</t>
+        </is>
+      </c>
+      <c r="H39" s="6" t="inlineStr">
         <is>
           <t>Текст есть</t>
         </is>
       </c>
-      <c r="H39" s="3" t="inlineStr">
+      <c r="I39" s="5" t="inlineStr">
         <is>
           <t>Требует правок</t>
         </is>
       </c>
-      <c r="I39" s="2" t="inlineStr">
-        <is>
-          <t>Нейтрально-негатив с зелёной иконкой успеха</t>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>Нейтрально-негатив с зелёной иконкой успеха (цвет/иконка)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I39"/>
+  <autoFilter ref="A1:J39"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2349,302 +2554,395 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B29"/>
+  <dimension ref="A1:B40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="78" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
-        <is>
-          <t>ГРУППЫ (по теме сообщения)</t>
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>ПРИНЦИП: язык определяется ВОРКГРУППОЙ, а не тем, что отрендерилось в макете.</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>Воркгруппа = страна + регулятор + язык. Поэтому язык отдельно не аудируем — он подставляется автоматически. Исключение: текст «вшит в код» — он воркгруппу игнорирует, это и есть единственный языковой дефект.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>ВОРКГРУППЫ</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>SIGAP_BRAZIL</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Бразилия, регулятор SIGAP → язык португальский (pt-BR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>NONE_MEXICO</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Мексика, без отдельного регулятора → язык испанский (es-MX)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>BCE</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Отдельная воркгруппа, не по схеме «страна» — уточнить у разработки</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Все</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Без фильтра по стране — показывается во всех странах (нужны все языки)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Все, кроме Бразилии</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Все страны, кроме SIGAP_BRAZIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>❓ уточнить</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Воркгруппа неизвестна (сообщения нет в дев-документации)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>ГРУППЫ (по теме)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
         <is>
           <t>Доступ и регуляторика</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
-        <is>
-          <t>Возраст, блокировки SIGAP, геолокация, согласие на cookie</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Возраст, блокировки SIGAP, геолокация, cookie</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>Верификация и безопасность</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>KYC, повторная верификация, проверка статуса, смена пароля</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>KYC, повторная верификация, статус, смена пароля</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>Ответственная игра</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
-        <is>
-          <t>Лимиты проигрышей/ставок, лимит игрового времени</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Лимиты проигрышей/ставок, лимит времени</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>Бонусы и промо</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
-        <is>
-          <t>Первый бонус, купоны, промокоды, выбор бонуса, выигрыши, реферал</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Бонусы, купоны, промокоды, выигрыши, реферал</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>Геймификация</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>Уровни, VIP-статус, карточки</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>Транзакции</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>Пополнение: успех и ошибка</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
         <is>
           <t>Игровой процесс</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>Демо-режим, бонусы в играх, баланс, фриспины, вейджер</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>Демо, бонусы в играх, баланс, фриспины, вейджер</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
         <is>
           <t>UI-действия</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
-        <is>
-          <t>Реакции на действия (избранное и т.п.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>Реакции на действия (избранное)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
         <is>
           <t>Системное / приложение</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>Обновления, блокировки доступа, технические ошибки</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>ВИДЫ (тип компонента — КАК показывается)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Обновления, доступ, технические ошибки</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>ВИДЫ (тип компонента)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
         <is>
           <t>Большое окно</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
-        <is>
-          <t>Модальное окно поверх экрана, с крестиком/кнопками</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>Модальное окно поверх экрана</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="inlineStr">
         <is>
           <t>Блокирующее окно</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>Окно без свободного закрытия — пока не выполнишь условие</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Окно без свободного закрытия</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
         <is>
           <t>Окно-событие</t>
         </is>
       </c>
-      <c r="B15" s="8" t="inlineStr">
-        <is>
-          <t>Всплывает само при событии (выигрыш, уровень, бонус)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr">
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>Всплывает само при событии</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
         <is>
           <t>Inline-баннер</t>
         </is>
       </c>
-      <c r="B16" s="8" t="inlineStr">
-        <is>
-          <t>Полоса внизу/вверху экрана, не перекрывает контент</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="7" t="inlineStr">
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>Полоса, не перекрывает контент</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr">
         <is>
           <t>Плашка (тост)</t>
         </is>
       </c>
-      <c r="B17" s="8" t="inlineStr">
-        <is>
-          <t>Маленькое сообщение, появляется ненадолго и исчезает</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>Маленькое сообщение, исчезает само</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="inlineStr">
         <is>
           <t>Алерт приложения</t>
         </is>
       </c>
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>Системное уведомление приложения (обновление, доступ)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>СТАТУС КОНТЕНТА (есть ли реальный текст)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="7" t="inlineStr">
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>Системное уведомление приложения</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>СТАТУС КОНТЕНТА</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
+          <t>i18n-ключ</t>
+        </is>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>Текст подставляется по воркгруппе → язык правильный автоматически. Нужно лишь запросить саму формулировку для ревью</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="10" t="inlineStr">
+        <is>
+          <t>Вшит в код</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>Текст прописан в коде → язык НЕ переключается по воркгруппе. Реальный языковой дефект, выносить в локализацию (разработка)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="inlineStr">
         <is>
           <t>Текст есть</t>
         </is>
       </c>
-      <c r="B21" s="8" t="inlineStr">
-        <is>
-          <t>Реальная формулировка известна — можно редактировать</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t>Нет текста (заглушка)</t>
-        </is>
-      </c>
-      <c r="B22" s="8" t="inlineStr">
-        <is>
-          <t>Вместо текста служебный код-ключ — нужен реальный текст от разработки</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="7" t="inlineStr">
-        <is>
-          <t>Вшит в код</t>
-        </is>
-      </c>
-      <c r="B23" s="8" t="inlineStr">
-        <is>
-          <t>Текст написан прямо в коде, переводится/правится только через разработку</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="7" t="inlineStr">
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>Формулировка известна, можно редактировать</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="10" t="inlineStr">
         <is>
           <t>Нет данных</t>
         </is>
       </c>
-      <c r="B24" s="8" t="inlineStr">
-        <is>
-          <t>Сообщение есть, но текста/кнопок в источниках нет</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="6" t="inlineStr">
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>Текста/кнопок в источниках нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="9" t="inlineStr">
         <is>
           <t>СТАТУС (что делать)</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="7" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="10" t="inlineStr">
         <is>
           <t>ОК</t>
         </is>
       </c>
-      <c r="B27" s="8" t="inlineStr">
-        <is>
-          <t>Проблем не видно, трогать не нужно</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="7" t="inlineStr">
+      <c r="B38" s="8" t="inlineStr">
+        <is>
+          <t>Проблем не видно</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="10" t="inlineStr">
         <is>
           <t>Требует правок</t>
         </is>
       </c>
-      <c r="B28" s="8" t="inlineStr">
-        <is>
-          <t>Видна проблема дизайна/контента (язык, цвет, формулировка) — зона дизайнера</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="7" t="inlineStr">
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t>Видна проблема (вшитый текст / цвет-иконка / формулировка / дубль)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="10" t="inlineStr">
         <is>
           <t>Уточнить у разработки</t>
         </is>
       </c>
-      <c r="B29" s="8" t="inlineStr">
-        <is>
-          <t>Не хватает данных, нужен запрос к команде</t>
+      <c r="B40" s="8" t="inlineStr">
+        <is>
+          <t>Не хватает данных (текста или воркгруппы)</t>
         </is>
       </c>
     </row>
@@ -2659,27 +2957,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B28"/>
+  <dimension ref="A1:B37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>По группам</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="9" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>Значение</t>
         </is>
       </c>
-      <c r="B2" s="9" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>Кол-во</t>
         </is>
@@ -2776,19 +3074,19 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>По видам</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>Значение</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>Кол-во</t>
         </is>
@@ -2855,19 +3153,19 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>По статусу (что делать)</t>
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>По воркгруппам</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="9" t="inlineStr">
+      <c r="A23" s="11" t="inlineStr">
         <is>
           <t>Значение</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B23" s="11" t="inlineStr">
         <is>
           <t>Кол-во</t>
         </is>
@@ -2876,37 +3174,116 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Требует правок</t>
+          <t>❓ уточнить</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Уточнить у разработки</t>
+          <t>Все</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>SIGAP_BRAZIL</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>NONE_MEXICO</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>BCE</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Все, кроме Бразилии</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>По статусу (что делать)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="11" t="inlineStr">
+        <is>
+          <t>Значение</t>
+        </is>
+      </c>
+      <c r="B32" s="11" t="inlineStr">
+        <is>
+          <t>Кол-во</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Требует правок</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Уточнить у разработки</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>ОК</t>
         </is>
       </c>
-      <c r="B26" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="6" t="inlineStr">
-        <is>
-          <t>ВСЕГО сообщений: 38</t>
+      <c r="B35" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="9" t="inlineStr">
+        <is>
+          <t>ВСЕГО: 38</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Re-pass all types: final-model component type + severity-by-meaning + Snackbar/Push split
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014BTMoKe4qeivFFNX4KkDkH
</commit_message>
<xml_diff>
--- a/_audit/Системные_сообщения_таблица.xlsx
+++ b/_audit/Системные_сообщения_таблица.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сводка" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Сообщения'!$A$1:$J$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Сообщения'!$A$1:$K$39</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,24 +31,27 @@
     </font>
     <font>
       <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <b val="1"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
     </font>
     <font>
       <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -73,6 +76,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DCE6F1"/>
       </patternFill>
     </fill>
     <fill>
@@ -107,7 +115,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -121,19 +129,22 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -499,19 +510,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J39"/>
+  <dimension ref="A1:K39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="44" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="46" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -527,40 +539,45 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Группа</t>
+          <t>Группа (тема)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Вид (тип компонента)</t>
+          <t>Тип (финальная модель)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Severity (по смыслу)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Когда показывается</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Воркгруппа (страна/регион)</t>
-        </is>
-      </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Ожидаемый язык (по воркгруппе)</t>
+          <t>Воркгруппа</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>Ожидаемый язык</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>Статус контента</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Статус (что делать)</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Комментарий</t>
         </is>
@@ -584,37 +601,42 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Большое окно</t>
+          <t>Dialog · обычный</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
           <t>Первый вход, возраст не подтверждён</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>SIGAP_BRAZIL</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Português (pt-BR)</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>i18n-ключ</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="J2" s="4" t="inlineStr">
         <is>
           <t>Уточнить у разработки</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>Текст локализуется по воркгруппе; запросить реальную формулировку</t>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Запросить реальную формулировку</t>
         </is>
       </c>
     </row>
@@ -636,37 +658,42 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Большое окно</t>
+          <t>Dialog · обычный</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Пришла команда блокировки от регулятора</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
+          <t>Команда блокировки от регулятора</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
           <t>SIGAP_BRAZIL</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Português (pt-BR)</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>i18n-ключ</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="J3" s="4" t="inlineStr">
         <is>
           <t>Уточнить у разработки</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>Запросить реальную формулировку</t>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Запросить формулировку</t>
         </is>
       </c>
     </row>
@@ -688,37 +715,42 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Блокирующее окно</t>
+          <t>Dialog · блокирующий</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
           <t>Заблокированный заходит на игру/спорт</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>SIGAP_BRAZIL</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Português (pt-BR)</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>i18n-ключ</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>Уточнить у разработки</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>Критично (окно без выхода); запросить выверенный текст</t>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Критично; запросить выверенный текст</t>
         </is>
       </c>
     </row>
@@ -740,37 +772,42 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Большое окно</t>
+          <t>Dialog · обычный</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Превышен платёжный лимит, не верифицирован</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
+          <t>Превышен платёжный лимит</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
           <t>NONE_MEXICO</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>Español (es-MX)</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Español</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>i18n-ключ</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t>Уточнить у разработки</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>Мало деталей по поведению; запросить текст</t>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Запросить текст и детали поведения</t>
         </is>
       </c>
     </row>
@@ -792,37 +829,42 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Большое окно</t>
+          <t>Dialog · обычный</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
           <t>Нужно заново подтвердить личность</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>SIGAP_BRAZIL</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Português (pt-BR)</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>i18n-ключ</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr">
+      <c r="J6" s="4" t="inlineStr">
         <is>
           <t>Уточнить у разработки</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>Запросить реальную формулировку</t>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Запросить формулировку</t>
         </is>
       </c>
     </row>
@@ -844,37 +886,42 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Большое окно</t>
+          <t>Dialog · блокирующий</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
           <t>Наиграно установленное время</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>SIGAP_BRAZIL</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>Português (pt-BR)</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>i18n-ключ</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="J7" s="4" t="inlineStr">
         <is>
           <t>Уточнить у разработки</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>Запросить реальную формулировку</t>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Запросить формулировку</t>
         </is>
       </c>
     </row>
@@ -896,37 +943,42 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Большое окно</t>
+          <t>Dialog · обычный</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
           <t>Вошёл, но не верифицирован</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>SIGAP_BRAZIL</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>Português (pt-BR)</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>i18n-ключ</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr">
+      <c r="J8" s="4" t="inlineStr">
         <is>
           <t>Уточнить у разработки</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>Многошаговый флоу — шаги и кнопки не ясны</t>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Шаги/кнопки не ясны</t>
         </is>
       </c>
     </row>
@@ -948,37 +1000,42 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Inline-баннер</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
+          <t>Banner</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>info</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Первый визит</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>BCE</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>❓ уточнить (BCE)</t>
-        </is>
-      </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>❓ уточнить</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
         <is>
           <t>Вшит в код</t>
         </is>
       </c>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="J9" s="6" t="inlineStr">
         <is>
           <t>Требует правок</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>Текст вшит в код → НЕ переключает язык по воркгруппе. Вынести в локализацию (задача разработки)</t>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Вшит в код → не локализуется по воркгруппе. Вынести в i18n</t>
         </is>
       </c>
     </row>
@@ -1000,37 +1057,42 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Большое окно</t>
+          <t>Dialog · обычный</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
           <t>Сразу после регистрации</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Все, кроме Бразилии</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>Все локали, кроме PT</t>
-        </is>
-      </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Все, кроме PT</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
         <is>
           <t>Вшит в код</t>
         </is>
       </c>
-      <c r="I10" s="5" t="inlineStr">
+      <c r="J10" s="6" t="inlineStr">
         <is>
           <t>Требует правок</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>Вшит в код → один язык на все страны. Вынести в локализацию. Плюс конкуренция окон после рег</t>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Вшит в код. Конкурирует с другими окнами после рег</t>
         </is>
       </c>
     </row>
@@ -1052,37 +1114,42 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Блокирующее окно</t>
+          <t>Dialog · блокирующий</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
           <t>Система требует сменить пароль</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Все</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>Все активные локали</t>
-        </is>
-      </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Все локали</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
         <is>
           <t>i18n-ключ</t>
         </is>
       </c>
-      <c r="I11" s="4" t="inlineStr">
+      <c r="J11" s="4" t="inlineStr">
         <is>
           <t>Уточнить у разработки</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>Запросить реальную формулировку</t>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Запросить формулировку</t>
         </is>
       </c>
     </row>
@@ -1104,37 +1171,42 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Большое окно</t>
+          <t>Dialog · обычный</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
           <t>После регистрации</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>SIGAP_BRAZIL</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>Português (pt-BR)</t>
-        </is>
-      </c>
-      <c r="H12" s="4" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
         <is>
           <t>Вшит в код</t>
         </is>
       </c>
-      <c r="I12" s="5" t="inlineStr">
+      <c r="J12" s="6" t="inlineStr">
         <is>
           <t>Требует правок</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>Вшит в код → не подхватит PT по воркгруппе. Вынести в локализацию</t>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Вшит в код → вынести в i18n</t>
         </is>
       </c>
     </row>
@@ -1156,37 +1228,42 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Блокирующее окно</t>
+          <t>Dialog · блокирующий</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
           <t>После верификации, если лимиты не заданы</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>SIGAP_BRAZIL</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>Português (pt-BR)</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
         <is>
           <t>i18n-ключ</t>
         </is>
       </c>
-      <c r="I13" s="4" t="inlineStr">
+      <c r="J13" s="4" t="inlineStr">
         <is>
           <t>Уточнить у разработки</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>Обязательное окно; запросить реальную формулировку</t>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Обязательное окно; запросить текст</t>
         </is>
       </c>
     </row>
@@ -1208,37 +1285,42 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Окно-событие</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
+          <t>Dialog · событие</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>Достигнут новый уровень</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>Все</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>Все активные локали</t>
-        </is>
-      </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Все локали</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>Вшит в код</t>
         </is>
       </c>
-      <c r="I14" s="5" t="inlineStr">
+      <c r="J14" s="6" t="inlineStr">
         <is>
           <t>Требует правок</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>Вшит в код → один язык на все страны. Дублирует «уровень» из M-09</t>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Вшит в код. Дублирует «уровень» из M-09</t>
         </is>
       </c>
     </row>
@@ -1260,37 +1342,42 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Окно-событие</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
+          <t>Dialog · событие</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>Апгрейд VIP</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>Все</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>Все активные локали</t>
-        </is>
-      </c>
-      <c r="H15" s="4" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Все локали</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
         <is>
           <t>Вшит в код</t>
         </is>
       </c>
-      <c r="I15" s="5" t="inlineStr">
+      <c r="J15" s="6" t="inlineStr">
         <is>
           <t>Требует правок</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>Вшит в код → вынести в локализацию</t>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Вшит в код</t>
         </is>
       </c>
     </row>
@@ -1312,37 +1399,42 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Окно-событие</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>Выигрыш по wager/фрибету/фриспину</t>
+          <t>Dialog · событие</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>success</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
+          <t>Выигрыш wager/фрибет/фриспин</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
           <t>Все</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>Все активные локали</t>
-        </is>
-      </c>
-      <c r="H16" s="4" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Все локали</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr">
         <is>
           <t>Вшит в код</t>
         </is>
       </c>
-      <c r="I16" s="5" t="inlineStr">
+      <c r="J16" s="6" t="inlineStr">
         <is>
           <t>Требует правок</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>Вшит в код → вынести в локализацию</t>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Вшит в код</t>
         </is>
       </c>
     </row>
@@ -1364,37 +1456,42 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Окно-событие</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
+          <t>Dialog · событие</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>Начисление за реферал</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>Все</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>Все активные локали</t>
-        </is>
-      </c>
-      <c r="H17" s="4" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Все локали</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
         <is>
           <t>Вшит в код</t>
         </is>
       </c>
-      <c r="I17" s="5" t="inlineStr">
+      <c r="J17" s="6" t="inlineStr">
         <is>
           <t>Требует правок</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>Вшит в код → вынести в локализацию</t>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Вшит в код</t>
         </is>
       </c>
     </row>
@@ -1416,37 +1513,42 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Окно-событие</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
+          <t>Dialog · событие</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>info</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Доступен бонус для активации</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>Все</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>Все активные локали</t>
-        </is>
-      </c>
-      <c r="H18" s="4" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Все локали</t>
+        </is>
+      </c>
+      <c r="I18" s="4" t="inlineStr">
         <is>
           <t>Вшит в код</t>
         </is>
       </c>
-      <c r="I18" s="5" t="inlineStr">
+      <c r="J18" s="6" t="inlineStr">
         <is>
           <t>Требует правок</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>Вшит в код → вынести в локализацию</t>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Вшит в код</t>
         </is>
       </c>
     </row>
@@ -1468,37 +1570,42 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Окно-событие</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
+          <t>Dialog · событие</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>Получена новая карточка</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>Все</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>Все активные локали</t>
-        </is>
-      </c>
-      <c r="H19" s="4" t="inlineStr">
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Все локали</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="inlineStr">
         <is>
           <t>Нет данных</t>
         </is>
       </c>
-      <c r="I19" s="4" t="inlineStr">
+      <c r="J19" s="4" t="inlineStr">
         <is>
           <t>Уточнить у разработки</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>Текст и кнопки в источниках не описаны</t>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Текст и кнопки не описаны</t>
         </is>
       </c>
     </row>
@@ -1520,37 +1627,42 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Окно-событие</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
+          <t>Dialog · событие</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>Успешно активирован промокод</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>Все</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>Все активные локали</t>
-        </is>
-      </c>
-      <c r="H20" s="4" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Все локали</t>
+        </is>
+      </c>
+      <c r="I20" s="4" t="inlineStr">
         <is>
           <t>Вшит в код</t>
         </is>
       </c>
-      <c r="I20" s="5" t="inlineStr">
+      <c r="J20" s="6" t="inlineStr">
         <is>
           <t>Требует правок</t>
         </is>
       </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>Вшит в код → вынести в локализацию</t>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Вшит в код</t>
         </is>
       </c>
     </row>
@@ -1572,37 +1684,42 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Окно-событие</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
+          <t>Dialog · обычный</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>Запуск игры без демо-режима</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="G21" s="2" t="inlineStr">
         <is>
           <t>Все</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>Все активные локали</t>
-        </is>
-      </c>
-      <c r="H21" s="4" t="inlineStr">
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Все локали</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="inlineStr">
         <is>
           <t>Вшит в код</t>
         </is>
       </c>
-      <c r="I21" s="5" t="inlineStr">
+      <c r="J21" s="6" t="inlineStr">
         <is>
           <t>Требует правок</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr">
-        <is>
-          <t>Вшит в код → вынести в локализацию. Встречается под двумя именами — возможно дубль</t>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Вшит в код. Два имени — возможно дубль</t>
         </is>
       </c>
     </row>
@@ -1624,37 +1741,42 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Алерт приложения</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>Доступно обновление</t>
+          <t>App alert → Dialog (блок.)</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>warning</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
+          <t>Доступно обязательное обновление</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
           <t>❓ уточнить</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>зависит от воркгруппы</t>
-        </is>
-      </c>
-      <c r="H22" s="6" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>зависит от ВГ</t>
+        </is>
+      </c>
+      <c r="I22" s="7" t="inlineStr">
         <is>
           <t>Текст есть</t>
         </is>
       </c>
-      <c r="I22" s="4" t="inlineStr">
+      <c r="J22" s="4" t="inlineStr">
         <is>
           <t>Уточнить у разработки</t>
         </is>
       </c>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>Плашки нет в дев-документации — подтвердить воркгруппу</t>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Подтвердить: блокирующее → Dialog. Воркгруппа неизвестна</t>
         </is>
       </c>
     </row>
@@ -1676,37 +1798,42 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Алерт приложения</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>Вышла новая версия</t>
+          <t>App alert → Banner</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>info</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
+          <t>Вышла новая версия (необязательно)</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
           <t>❓ уточнить</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr">
-        <is>
-          <t>зависит от воркгруппы</t>
-        </is>
-      </c>
-      <c r="H23" s="6" t="inlineStr">
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>зависит от ВГ</t>
+        </is>
+      </c>
+      <c r="I23" s="7" t="inlineStr">
         <is>
           <t>Текст есть</t>
         </is>
       </c>
-      <c r="I23" s="4" t="inlineStr">
+      <c r="J23" s="4" t="inlineStr">
         <is>
           <t>Уточнить у разработки</t>
         </is>
       </c>
-      <c r="J23" s="2" t="inlineStr">
-        <is>
-          <t>Плашки нет в дев-документации — подтвердить воркгруппу</t>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>Мягкое → Banner. Воркгруппа неизвестна</t>
         </is>
       </c>
     </row>
@@ -1728,37 +1855,42 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Алерт приложения</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>Пользователь заблокирован/не зарегистрирован</t>
+          <t>Dialog · блокирующий</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
+          <t>Пользователь заблокирован</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
           <t>❓ уточнить</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>зависит от воркгруппы</t>
-        </is>
-      </c>
-      <c r="H24" s="6" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>зависит от ВГ</t>
+        </is>
+      </c>
+      <c r="I24" s="7" t="inlineStr">
         <is>
           <t>Текст есть</t>
         </is>
       </c>
-      <c r="I24" s="4" t="inlineStr">
+      <c r="J24" s="4" t="inlineStr">
         <is>
           <t>Уточнить у разработки</t>
         </is>
       </c>
-      <c r="J24" s="2" t="inlineStr">
-        <is>
-          <t>Плашки нет в дев-документации — подтвердить воркгруппу</t>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>Воркгруппа неизвестна</t>
         </is>
       </c>
     </row>
@@ -1780,37 +1912,42 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Плашка (тост)</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
+          <t>Snackbar</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
         <is>
           <t>Депозит прошёл успешно</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr">
+      <c r="G25" s="2" t="inlineStr">
         <is>
           <t>❓ уточнить</t>
         </is>
       </c>
-      <c r="G25" s="2" t="inlineStr">
-        <is>
-          <t>зависит от воркгруппы</t>
-        </is>
-      </c>
-      <c r="H25" s="6" t="inlineStr">
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>зависит от ВГ</t>
+        </is>
+      </c>
+      <c r="I25" s="7" t="inlineStr">
         <is>
           <t>Текст есть</t>
         </is>
       </c>
-      <c r="I25" s="5" t="inlineStr">
+      <c r="J25" s="6" t="inlineStr">
         <is>
           <t>Требует правок</t>
         </is>
       </c>
-      <c r="J25" s="2" t="inlineStr">
-        <is>
-          <t>Успех помечен оранжевой иконкой предупреждения (цвет/иконка)</t>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>SEVERITY НЕВЕРНО: success, а иконка оранжевая info/warning</t>
         </is>
       </c>
     </row>
@@ -1832,37 +1969,42 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Плашка (тост)</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
+          <t>Snackbar</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>Добавление в избранное</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>❓ уточнить</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
-        <is>
-          <t>зависит от воркгруппы</t>
-        </is>
-      </c>
-      <c r="H26" s="6" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>зависит от ВГ</t>
+        </is>
+      </c>
+      <c r="I26" s="7" t="inlineStr">
         <is>
           <t>Текст есть</t>
         </is>
       </c>
-      <c r="I26" s="6" t="inlineStr">
-        <is>
-          <t>ОК</t>
-        </is>
-      </c>
-      <c r="J26" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="J26" s="6" t="inlineStr">
+        <is>
+          <t>Требует правок</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>SEVERITY НЕВЕРНО: success, а иконка оранжевая info</t>
         </is>
       </c>
     </row>
@@ -1884,37 +2026,42 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Плашка (тост)</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
+          <t>Snackbar</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>info</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
         <is>
           <t>Удаление из избранного</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
+      <c r="G27" s="2" t="inlineStr">
         <is>
           <t>❓ уточнить</t>
         </is>
       </c>
-      <c r="G27" s="2" t="inlineStr">
-        <is>
-          <t>зависит от воркгруппы</t>
-        </is>
-      </c>
-      <c r="H27" s="6" t="inlineStr">
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>зависит от ВГ</t>
+        </is>
+      </c>
+      <c r="I27" s="7" t="inlineStr">
         <is>
           <t>Текст есть</t>
         </is>
       </c>
-      <c r="I27" s="5" t="inlineStr">
+      <c r="J27" s="6" t="inlineStr">
         <is>
           <t>Требует правок</t>
         </is>
       </c>
-      <c r="J27" s="2" t="inlineStr">
-        <is>
-          <t>Формулировка-команда вместо факта («Удалено из избранного»)</t>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>Формулировка-команда вместо факта («Удалено»)</t>
         </is>
       </c>
     </row>
@@ -1936,37 +2083,42 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Плашка (тост)</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
+          <t>Snackbar</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>Включены инструменты геолокации</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>❓ уточнить</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>зависит от воркгруппы</t>
-        </is>
-      </c>
-      <c r="H28" s="6" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>зависит от ВГ</t>
+        </is>
+      </c>
+      <c r="I28" s="7" t="inlineStr">
         <is>
           <t>Текст есть</t>
         </is>
       </c>
-      <c r="I28" s="6" t="inlineStr">
+      <c r="J28" s="7" t="inlineStr">
         <is>
           <t>ОК</t>
         </is>
       </c>
-      <c r="J28" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>Severity (warning) и иконка совпадают</t>
         </is>
       </c>
     </row>
@@ -1988,37 +2140,42 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Плашка (тост)</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
+          <t>Snackbar</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
         <is>
           <t>Сбой обработки запроса</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr">
+      <c r="G29" s="2" t="inlineStr">
         <is>
           <t>❓ уточнить</t>
         </is>
       </c>
-      <c r="G29" s="2" t="inlineStr">
-        <is>
-          <t>зависит от воркгруппы</t>
-        </is>
-      </c>
-      <c r="H29" s="6" t="inlineStr">
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>зависит от ВГ</t>
+        </is>
+      </c>
+      <c r="I29" s="7" t="inlineStr">
         <is>
           <t>Текст есть</t>
         </is>
       </c>
-      <c r="I29" s="5" t="inlineStr">
+      <c r="J29" s="6" t="inlineStr">
         <is>
           <t>Требует правок</t>
         </is>
       </c>
-      <c r="J29" s="2" t="inlineStr">
-        <is>
-          <t>Помечено как предупреждение, хотя это ошибка (цвет/иконка)</t>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>SEVERITY НЕВЕРНО: error, а помечено warning</t>
         </is>
       </c>
     </row>
@@ -2040,37 +2197,42 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Плашка (тост)</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
+          <t>Snackbar</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Сбой депозита</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>❓ уточнить</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t>зависит от воркгруппы</t>
-        </is>
-      </c>
-      <c r="H30" s="6" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>зависит от ВГ</t>
+        </is>
+      </c>
+      <c r="I30" s="7" t="inlineStr">
         <is>
           <t>Текст есть</t>
         </is>
       </c>
-      <c r="I30" s="6" t="inlineStr">
+      <c r="J30" s="7" t="inlineStr">
         <is>
           <t>ОК</t>
         </is>
       </c>
-      <c r="J30" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>Severity (error, красный ✕) корректно</t>
         </is>
       </c>
     </row>
@@ -2092,37 +2254,42 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Плашка (тост)</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
+          <t>Snackbar</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
         <is>
           <t>Сбой записи в розыгрыш</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr">
+      <c r="G31" s="2" t="inlineStr">
         <is>
           <t>❓ уточнить</t>
         </is>
       </c>
-      <c r="G31" s="2" t="inlineStr">
-        <is>
-          <t>зависит от воркгруппы</t>
-        </is>
-      </c>
-      <c r="H31" s="6" t="inlineStr">
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>зависит от ВГ</t>
+        </is>
+      </c>
+      <c r="I31" s="7" t="inlineStr">
         <is>
           <t>Текст есть</t>
         </is>
       </c>
-      <c r="I31" s="6" t="inlineStr">
+      <c r="J31" s="7" t="inlineStr">
         <is>
           <t>ОК</t>
         </is>
       </c>
-      <c r="J31" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>Severity (error, красный ✕) корректно</t>
         </is>
       </c>
     </row>
@@ -2144,37 +2311,42 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Плашка (тост)</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
+          <t>Push (уточнить)</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>Достигнут лимит проигрышей</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>❓ уточнить</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
-        <is>
-          <t>зависит от воркгруппы</t>
-        </is>
-      </c>
-      <c r="H32" s="6" t="inlineStr">
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>зависит от ВГ</t>
+        </is>
+      </c>
+      <c r="I32" s="7" t="inlineStr">
         <is>
           <t>Текст есть</t>
         </is>
       </c>
-      <c r="I32" s="5" t="inlineStr">
+      <c r="J32" s="6" t="inlineStr">
         <is>
           <t>Требует правок</t>
         </is>
       </c>
-      <c r="J32" s="2" t="inlineStr">
-        <is>
-          <t>Та же тема, что окно лимитов — дублирование канала, свести тон</t>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>НЕ error: это уведомление RG (warning). Лого BB+точка → похоже push, уточнить</t>
         </is>
       </c>
     </row>
@@ -2196,37 +2368,42 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Плашка (тост)</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
+          <t>Push (уточнить)</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
         <is>
           <t>Достигнут лимит ставок</t>
         </is>
       </c>
-      <c r="F33" s="2" t="inlineStr">
+      <c r="G33" s="2" t="inlineStr">
         <is>
           <t>❓ уточнить</t>
         </is>
       </c>
-      <c r="G33" s="2" t="inlineStr">
-        <is>
-          <t>зависит от воркгруппы</t>
-        </is>
-      </c>
-      <c r="H33" s="6" t="inlineStr">
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>зависит от ВГ</t>
+        </is>
+      </c>
+      <c r="I33" s="7" t="inlineStr">
         <is>
           <t>Текст есть</t>
         </is>
       </c>
-      <c r="I33" s="5" t="inlineStr">
+      <c r="J33" s="6" t="inlineStr">
         <is>
           <t>Требует правок</t>
         </is>
       </c>
-      <c r="J33" s="2" t="inlineStr">
-        <is>
-          <t>Та же тема, что окно лимитов — дублирование канала, свести тон</t>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>НЕ error: уведомление RG (warning). BB+точка → push, уточнить</t>
         </is>
       </c>
     </row>
@@ -2248,37 +2425,42 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Плашка (тост)</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
+          <t>Push (уточнить)</t>
+        </is>
+      </c>
+      <c r="E34" s="6" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>Бонус нельзя применить к спорту</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>❓ уточнить</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr">
-        <is>
-          <t>зависит от воркгруппы</t>
-        </is>
-      </c>
-      <c r="H34" s="6" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>зависит от ВГ</t>
+        </is>
+      </c>
+      <c r="I34" s="7" t="inlineStr">
         <is>
           <t>Текст есть</t>
         </is>
       </c>
-      <c r="I34" s="6" t="inlineStr">
-        <is>
-          <t>ОК</t>
-        </is>
-      </c>
-      <c r="J34" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="J34" s="6" t="inlineStr">
+        <is>
+          <t>Требует правок</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>НЕ error: ограничение (warning). BB+точка → push, уточнить</t>
         </is>
       </c>
     </row>
@@ -2290,7 +2472,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>«Недостаточно средств, пополните баланс»</t>
+          <t>«Недостаточно средств»</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -2300,37 +2482,42 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Плашка (тост)</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
+          <t>Snackbar</t>
+        </is>
+      </c>
+      <c r="E35" s="6" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
         <is>
           <t>Не хватает денег для игры</t>
         </is>
       </c>
-      <c r="F35" s="2" t="inlineStr">
+      <c r="G35" s="2" t="inlineStr">
         <is>
           <t>❓ уточнить</t>
         </is>
       </c>
-      <c r="G35" s="2" t="inlineStr">
-        <is>
-          <t>зависит от воркгруппы</t>
-        </is>
-      </c>
-      <c r="H35" s="6" t="inlineStr">
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>зависит от ВГ</t>
+        </is>
+      </c>
+      <c r="I35" s="7" t="inlineStr">
         <is>
           <t>Текст есть</t>
         </is>
       </c>
-      <c r="I35" s="5" t="inlineStr">
+      <c r="J35" s="6" t="inlineStr">
         <is>
           <t>Требует правок</t>
         </is>
       </c>
-      <c r="J35" s="2" t="inlineStr">
-        <is>
-          <t>Негатив с зелёной иконкой успеха (цвет/иконка)</t>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>SEVERITY НЕВЕРНО: негатив с зелёной success-иконкой</t>
         </is>
       </c>
     </row>
@@ -2352,37 +2539,42 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Плашка (тост)</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
+          <t>Snackbar</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>Не удалось активировать бонус</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>❓ уточнить</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
-        <is>
-          <t>зависит от воркгруппы</t>
-        </is>
-      </c>
-      <c r="H36" s="6" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>зависит от ВГ</t>
+        </is>
+      </c>
+      <c r="I36" s="7" t="inlineStr">
         <is>
           <t>Текст есть</t>
         </is>
       </c>
-      <c r="I36" s="6" t="inlineStr">
+      <c r="J36" s="7" t="inlineStr">
         <is>
           <t>ОК</t>
         </is>
       </c>
-      <c r="J36" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>Severity (error, красный ✕) корректно</t>
         </is>
       </c>
     </row>
@@ -2404,37 +2596,42 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Плашка (тост)</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
+          <t>Snackbar</t>
+        </is>
+      </c>
+      <c r="E37" s="6" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
         <is>
           <t>Фриспины уже активны</t>
         </is>
       </c>
-      <c r="F37" s="2" t="inlineStr">
+      <c r="G37" s="2" t="inlineStr">
         <is>
           <t>❓ уточнить</t>
         </is>
       </c>
-      <c r="G37" s="2" t="inlineStr">
-        <is>
-          <t>зависит от воркгруппы</t>
-        </is>
-      </c>
-      <c r="H37" s="6" t="inlineStr">
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>зависит от ВГ</t>
+        </is>
+      </c>
+      <c r="I37" s="7" t="inlineStr">
         <is>
           <t>Текст есть</t>
         </is>
       </c>
-      <c r="I37" s="6" t="inlineStr">
-        <is>
-          <t>ОК</t>
-        </is>
-      </c>
-      <c r="J37" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="J37" s="6" t="inlineStr">
+        <is>
+          <t>Требует правок</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>SEVERITY: это info/warning, а иконка error-красная</t>
         </is>
       </c>
     </row>
@@ -2456,37 +2653,42 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Плашка (тост)</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
+          <t>Push (уточнить)</t>
+        </is>
+      </c>
+      <c r="E38" s="6" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>Сумма ставки не равна фрибету</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>❓ уточнить</t>
         </is>
       </c>
-      <c r="G38" s="2" t="inlineStr">
-        <is>
-          <t>зависит от воркгруппы</t>
-        </is>
-      </c>
-      <c r="H38" s="6" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>зависит от ВГ</t>
+        </is>
+      </c>
+      <c r="I38" s="7" t="inlineStr">
         <is>
           <t>Текст есть</t>
         </is>
       </c>
-      <c r="I38" s="6" t="inlineStr">
-        <is>
-          <t>ОК</t>
-        </is>
-      </c>
-      <c r="J38" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="J38" s="6" t="inlineStr">
+        <is>
+          <t>Требует правок</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>Подсказка (warning), не error. BB+точка → push, уточнить</t>
         </is>
       </c>
     </row>
@@ -2508,42 +2710,47 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Плашка (тост)</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
+          <t>Snackbar</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>info</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
         <is>
           <t>Ставка не засчитывается в вейджер</t>
         </is>
       </c>
-      <c r="F39" s="2" t="inlineStr">
+      <c r="G39" s="2" t="inlineStr">
         <is>
           <t>❓ уточнить</t>
         </is>
       </c>
-      <c r="G39" s="2" t="inlineStr">
-        <is>
-          <t>зависит от воркгруппы</t>
-        </is>
-      </c>
-      <c r="H39" s="6" t="inlineStr">
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>зависит от ВГ</t>
+        </is>
+      </c>
+      <c r="I39" s="7" t="inlineStr">
         <is>
           <t>Текст есть</t>
         </is>
       </c>
-      <c r="I39" s="5" t="inlineStr">
+      <c r="J39" s="6" t="inlineStr">
         <is>
           <t>Требует правок</t>
         </is>
       </c>
-      <c r="J39" s="2" t="inlineStr">
-        <is>
-          <t>Нейтрально-негатив с зелёной иконкой успеха (цвет/иконка)</t>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>SEVERITY НЕВЕРНО: нейтральный факт (info) с зелёной success-иконкой</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J39"/>
+  <autoFilter ref="A1:K39"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2554,395 +2761,218 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B40"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="78" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="80" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
-        <is>
-          <t>ПРИНЦИП: язык определяется ВОРКГРУППОЙ, а не тем, что отрендерилось в макете.</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="8" t="inlineStr">
-        <is>
-          <t>Воркгруппа = страна + регулятор + язык. Поэтому язык отдельно не аудируем — он подставляется автоматически. Исключение: текст «вшит в код» — он воркгруппу игнорирует, это и есть единственный языковой дефект.</t>
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>ВАЖНО: severity проставлен ПО СМЫСЛУ, а не как на Figma-борде (там он часто неверный).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>ТИП (финальная модель)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
-        <is>
-          <t>ВОРКГРУППЫ</t>
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Dialog · обычный</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>Окно по центру, закрывается крестиком/кнопкой</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t>SIGAP_BRAZIL</t>
-        </is>
-      </c>
-      <c r="B5" s="8" t="inlineStr">
-        <is>
-          <t>Бразилия, регулятор SIGAP → язык португальский (pt-BR)</t>
+          <t>Dialog · блокирующий</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>Окно по центру без свободного закрытия (регуляторика, безопасность)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
         <is>
-          <t>NONE_MEXICO</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>Мексика, без отдельного регулятора → язык испанский (es-MX)</t>
+          <t>Dialog · событие</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>Окно по центру, всплывает само по реалтайм-событию (поздравление)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>BCE</t>
-        </is>
-      </c>
-      <c r="B7" s="8" t="inlineStr">
-        <is>
-          <t>Отдельная воркгруппа, не по схеме «страна» — уточнить у разработки</t>
+          <t>Bottom sheet</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Панель снизу (выбор/форма/промо)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
         <is>
-          <t>Все</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>Без фильтра по стране — показывается во всех странах (нужны все языки)</t>
+          <t>Snackbar</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>Плашка, сама исчезает, обратная связь на действие</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Все, кроме Бразилии</t>
-        </is>
-      </c>
-      <c r="B9" s="8" t="inlineStr">
-        <is>
-          <t>Все страны, кроме SIGAP_BRAZIL</t>
+          <t>Banner</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>Полоса-уведомление в странице, не перекрывает</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>❓ уточнить</t>
-        </is>
-      </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>Воркгруппа неизвестна (сообщения нет в дев-документации)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr">
-        <is>
-          <t>ГРУППЫ (по теме)</t>
+          <t>Push (уточнить)</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>Карточки с лого BB и красной точкой — похоже на push/инбокс, НЕ снекбар. Подтвердить у разработки</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>App alert → …</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>«Алерт приложения» не отдельный тип: блокирующий → Dialog, мягкий → Banner</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
-        <is>
-          <t>Доступ и регуляторика</t>
-        </is>
-      </c>
-      <c r="B13" s="8" t="inlineStr">
-        <is>
-          <t>Возраст, блокировки SIGAP, геолокация, cookie</t>
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>SEVERITY (по смыслу)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>Верификация и безопасность</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>KYC, повторная верификация, статус, смена пароля</t>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>Действие выполнено / положительное событие → зелёный ✓</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>Ответственная игра</t>
-        </is>
-      </c>
-      <c r="B15" s="8" t="inlineStr">
-        <is>
-          <t>Лимиты проигрышей/ставок, лимит времени</t>
+          <t>info</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>Нейтральный факт без оценки → нейтральный/синий</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Бонусы и промо</t>
-        </is>
-      </c>
-      <c r="B16" s="8" t="inlineStr">
-        <is>
-          <t>Бонусы, купоны, промокоды, выигрыши, реферал</t>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>Внимание/ограничение, но не сбой (лимит достигнут, гео) → оранжевый</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>Геймификация</t>
-        </is>
-      </c>
-      <c r="B17" s="8" t="inlineStr">
-        <is>
-          <t>Уровни, VIP-статус, карточки</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="10" t="inlineStr">
-        <is>
-          <t>Транзакции</t>
-        </is>
-      </c>
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>Пополнение: успех и ошибка</t>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>Сбой или отказ, что-то не выполнилось (депозит не прошёл) → красный ✕</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr">
-        <is>
-          <t>Игровой процесс</t>
-        </is>
-      </c>
-      <c r="B19" s="8" t="inlineStr">
-        <is>
-          <t>Демо, бонусы в играх, баланс, фриспины, вейджер</t>
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>СТАТУС (что делать)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="10" t="inlineStr">
         <is>
-          <t>UI-действия</t>
-        </is>
-      </c>
-      <c r="B20" s="8" t="inlineStr">
-        <is>
-          <t>Реакции на действия (избранное)</t>
+          <t>ОК</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Тип и severity корректны</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
         <is>
-          <t>Системное / приложение</t>
-        </is>
-      </c>
-      <c r="B21" s="8" t="inlineStr">
-        <is>
-          <t>Обновления, доступ, технические ошибки</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="9" t="inlineStr">
-        <is>
-          <t>ВИДЫ (тип компонента)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="10" t="inlineStr">
-        <is>
-          <t>Большое окно</t>
-        </is>
-      </c>
-      <c r="B24" s="8" t="inlineStr">
-        <is>
-          <t>Модальное окно поверх экрана</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="10" t="inlineStr">
-        <is>
-          <t>Блокирующее окно</t>
-        </is>
-      </c>
-      <c r="B25" s="8" t="inlineStr">
-        <is>
-          <t>Окно без свободного закрытия</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="10" t="inlineStr">
-        <is>
-          <t>Окно-событие</t>
-        </is>
-      </c>
-      <c r="B26" s="8" t="inlineStr">
-        <is>
-          <t>Всплывает само при событии</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="10" t="inlineStr">
-        <is>
-          <t>Inline-баннер</t>
-        </is>
-      </c>
-      <c r="B27" s="8" t="inlineStr">
-        <is>
-          <t>Полоса, не перекрывает контент</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="10" t="inlineStr">
-        <is>
-          <t>Плашка (тост)</t>
-        </is>
-      </c>
-      <c r="B28" s="8" t="inlineStr">
-        <is>
-          <t>Маленькое сообщение, исчезает само</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="10" t="inlineStr">
-        <is>
-          <t>Алерт приложения</t>
-        </is>
-      </c>
-      <c r="B29" s="8" t="inlineStr">
-        <is>
-          <t>Системное уведомление приложения</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="9" t="inlineStr">
-        <is>
-          <t>СТАТУС КОНТЕНТА</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="10" t="inlineStr">
-        <is>
-          <t>i18n-ключ</t>
-        </is>
-      </c>
-      <c r="B32" s="8" t="inlineStr">
-        <is>
-          <t>Текст подставляется по воркгруппе → язык правильный автоматически. Нужно лишь запросить саму формулировку для ревью</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="10" t="inlineStr">
-        <is>
-          <t>Вшит в код</t>
-        </is>
-      </c>
-      <c r="B33" s="8" t="inlineStr">
-        <is>
-          <t>Текст прописан в коде → язык НЕ переключается по воркгруппе. Реальный языковой дефект, выносить в локализацию (разработка)</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="10" t="inlineStr">
-        <is>
-          <t>Текст есть</t>
-        </is>
-      </c>
-      <c r="B34" s="8" t="inlineStr">
-        <is>
-          <t>Формулировка известна, можно редактировать</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="10" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="B35" s="8" t="inlineStr">
-        <is>
-          <t>Текста/кнопок в источниках нет</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="9" t="inlineStr">
-        <is>
-          <t>СТАТУС (что делать)</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="10" t="inlineStr">
-        <is>
-          <t>ОК</t>
-        </is>
-      </c>
-      <c r="B38" s="8" t="inlineStr">
-        <is>
-          <t>Проблем не видно</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="10" t="inlineStr">
-        <is>
           <t>Требует правок</t>
         </is>
       </c>
-      <c r="B39" s="8" t="inlineStr">
-        <is>
-          <t>Видна проблема (вшитый текст / цвет-иконка / формулировка / дубль)</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="10" t="inlineStr">
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Неверный severity / вшитый текст / формулировка / канал</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
         <is>
           <t>Уточнить у разработки</t>
         </is>
       </c>
-      <c r="B40" s="8" t="inlineStr">
-        <is>
-          <t>Не хватает данных (текста или воркгруппы)</t>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>Не хватает текста или воркгруппы</t>
         </is>
       </c>
     </row>
@@ -2957,27 +2987,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B37"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
-          <t>По группам</t>
+          <t>По типу</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>Значение</t>
         </is>
       </c>
-      <c r="B2" s="11" t="inlineStr">
+      <c r="B2" s="12" t="inlineStr">
         <is>
           <t>Кол-во</t>
         </is>
@@ -2986,47 +3016,47 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Бонусы и промо</t>
+          <t>Snackbar</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Игровой процесс</t>
+          <t>Dialog · обычный</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Доступ и регуляторика</t>
+          <t>Dialog · событие</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Верификация и безопасность</t>
+          <t>Dialog · блокирующий</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Ответственная игра</t>
+          <t>Push (уточнить)</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -3036,76 +3066,76 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Системное / приложение</t>
+          <t>Banner</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Геймификация</t>
+          <t>App alert → Dialog (блок.)</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Транзакции</t>
+          <t>App alert → Banner</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>UI-действия</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>2</v>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>По severity (по смыслу)</t>
+        </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>По видам</t>
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>Значение</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>Кол-во</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="inlineStr">
-        <is>
-          <t>Значение</t>
-        </is>
-      </c>
-      <c r="B14" s="11" t="inlineStr">
-        <is>
-          <t>Кол-во</t>
-        </is>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Плашка (тост)</t>
+          <t>warning</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Большое окно</t>
+          <t>success</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -3115,173 +3145,74 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Окно-событие</t>
+          <t>info</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Блокирующее окно</t>
+          <t>error</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Алерт приложения</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Inline-баннер</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>1</v>
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>По статусу (что делать)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>Значение</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>Кол-во</t>
+        </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="9" t="inlineStr">
-        <is>
-          <t>По воркгруппам</t>
-        </is>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Требует правок</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="11" t="inlineStr">
-        <is>
-          <t>Значение</t>
-        </is>
-      </c>
-      <c r="B23" s="11" t="inlineStr">
-        <is>
-          <t>Кол-во</t>
-        </is>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Уточнить у разработки</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>❓ уточнить</t>
+          <t>ОК</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Все</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>SIGAP_BRAZIL</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>NONE_MEXICO</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>BCE</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Все, кроме Бразилии</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="9" t="inlineStr">
-        <is>
-          <t>По статусу (что делать)</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="11" t="inlineStr">
-        <is>
-          <t>Значение</t>
-        </is>
-      </c>
-      <c r="B32" s="11" t="inlineStr">
-        <is>
-          <t>Кол-во</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Требует правок</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Уточнить у разработки</t>
-        </is>
-      </c>
-      <c r="B34" t="n">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>ОК</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="9" t="inlineStr">
+      <c r="A26" s="9" t="inlineStr">
         <is>
           <t>ВСЕГО: 38</t>
         </is>

</xml_diff>